<commit_message>
fixing labels on unfolding angles
</commit_message>
<xml_diff>
--- a/notes/LIBRA-I Unfolding Angles.xlsx
+++ b/notes/LIBRA-I Unfolding Angles.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WireDrive\Desktop\LIBRA-I\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WireDrive\Desktop\LIBRA-II\Software\LIBRA-II-App\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34F892E5-ED05-4B7F-A744-9C6FF3C2108D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D5722D5-35E8-428A-8A40-27F442D3D2F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{B4EF7078-C578-406F-A6BE-9F7C8010B763}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -47,19 +46,19 @@
     <t>J3</t>
   </si>
   <si>
-    <t>J4</t>
-  </si>
-  <si>
-    <t>J5</t>
-  </si>
-  <si>
-    <t>Pose 1</t>
-  </si>
-  <si>
-    <t>Pose 2</t>
-  </si>
-  <si>
-    <t>Pose 3</t>
+    <t>Step 1</t>
+  </si>
+  <si>
+    <t>Step 2</t>
+  </si>
+  <si>
+    <t>Step 3</t>
+  </si>
+  <si>
+    <t>Step 4</t>
+  </si>
+  <si>
+    <t>Step 5</t>
   </si>
 </sst>
 </file>
@@ -566,24 +565,24 @@
   <sheetData>
     <row r="1" spans="1:6" ht="18">
       <c r="B1" s="7" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="24" customHeight="1">
       <c r="A2" s="10" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B2" s="1">
         <v>0</v>
@@ -603,7 +602,7 @@
     </row>
     <row r="3" spans="1:6" ht="24" customHeight="1">
       <c r="A3" s="11" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B3" s="4">
         <v>0</v>
@@ -623,7 +622,7 @@
     </row>
     <row r="4" spans="1:6" ht="24" customHeight="1">
       <c r="A4" s="10" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="B4" s="1">
         <v>-150</v>

</xml_diff>

<commit_message>
updating unfolding angles with lessons learned with Goto-san
</commit_message>
<xml_diff>
--- a/notes/LIBRA-I Unfolding Angles.xlsx
+++ b/notes/LIBRA-I Unfolding Angles.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WireDrive\Desktop\LIBRA-II\Software\LIBRA-II-App\notes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brice.c.aa\Desktop\Projects\LIBRA-II\Software\LIBRA-I_App\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D5722D5-35E8-428A-8A40-27F442D3D2F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04D289FB-4799-4FDF-BB68-817C2A878953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{B4EF7078-C578-406F-A6BE-9F7C8010B763}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4EF7078-C578-406F-A6BE-9F7C8010B763}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>J1</t>
   </si>
@@ -59,13 +59,69 @@
   </si>
   <si>
     <t>Step 5</t>
+  </si>
+  <si>
+    <t>Pitch</t>
+  </si>
+  <si>
+    <t>Roll</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  0*</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">* At </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Pitch = 25 deg</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ENABLE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> water system</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -75,15 +131,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="6"/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="128"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
+      <sz val="6"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="128"/>
@@ -97,8 +152,31 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -123,8 +201,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCCCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -133,24 +217,35 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -161,9 +256,7 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -173,19 +266,10 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -194,10 +278,21 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
+      <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -206,42 +301,57 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -249,6 +359,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFCCCC"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -557,91 +672,144 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FB34EA6-0AD0-4819-861A-7A834B965178}">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.109375" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" style="7" customWidth="1"/>
+    <col min="2" max="16384" width="9.140625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18">
-      <c r="B1" s="7" t="s">
+    <row r="1" spans="1:6" ht="18.75">
+      <c r="B1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="24" customHeight="1">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="8">
         <v>0</v>
       </c>
-      <c r="B2" s="1">
+      <c r="C2" s="8">
         <v>0</v>
       </c>
-      <c r="C2" s="2">
-        <v>60</v>
-      </c>
-      <c r="D2" s="2">
-        <v>120</v>
-      </c>
-      <c r="E2" s="2">
-        <v>170</v>
-      </c>
-      <c r="F2" s="3">
-        <v>170</v>
+      <c r="D2" s="8">
+        <v>0</v>
+      </c>
+      <c r="E2" s="8">
+        <v>0</v>
+      </c>
+      <c r="F2" s="9">
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="24" customHeight="1">
-      <c r="A3" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4">
-        <v>0</v>
-      </c>
-      <c r="C3" s="5">
-        <v>-130</v>
-      </c>
-      <c r="D3" s="5">
-        <v>-170</v>
-      </c>
-      <c r="E3" s="5">
-        <v>-170</v>
-      </c>
-      <c r="F3" s="6">
-        <v>-170</v>
+      <c r="A3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="10">
+        <v>90</v>
+      </c>
+      <c r="C3" s="10">
+        <v>80</v>
+      </c>
+      <c r="D3" s="10">
+        <v>80</v>
+      </c>
+      <c r="E3" s="10">
+        <v>70</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="24" customHeight="1">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="12">
+        <v>0</v>
+      </c>
+      <c r="C4" s="12">
+        <v>60</v>
+      </c>
+      <c r="D4" s="12">
+        <v>120</v>
+      </c>
+      <c r="E4" s="12">
+        <v>160</v>
+      </c>
+      <c r="F4" s="13">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="24" customHeight="1">
+      <c r="A5" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="10">
+        <v>0</v>
+      </c>
+      <c r="C5" s="10">
+        <v>-130</v>
+      </c>
+      <c r="D5" s="10">
+        <v>-170</v>
+      </c>
+      <c r="E5" s="10">
+        <v>-170</v>
+      </c>
+      <c r="F5" s="11">
+        <v>-160</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="24" customHeight="1">
+      <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B6" s="14">
         <v>-150</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C6" s="14">
         <v>-90</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D6" s="14">
         <v>-45</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E6" s="14">
         <v>-45</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F6" s="15">
         <v>-170</v>
       </c>
+    </row>
+    <row r="8" spans="1:6" ht="18.75" customHeight="1">
+      <c r="B8" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="1"/>
+  <mergeCells count="1">
+    <mergeCell ref="B8:F8"/>
+  </mergeCells>
+  <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
added colors for ease of differentiating changing angles
</commit_message>
<xml_diff>
--- a/notes/LIBRA-I Unfolding Angles.xlsx
+++ b/notes/LIBRA-I Unfolding Angles.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brice.c.aa\Desktop\Projects\LIBRA-II\Software\LIBRA-I_App\notes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brice\Desktop\Projects\LIBRA-II\Software\LIBRA-I_App\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04D289FB-4799-4FDF-BB68-817C2A878953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D46F624-5C26-49A5-A795-7EBDAFC47528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4EF7078-C578-406F-A6BE-9F7C8010B763}"/>
   </bookViews>
@@ -121,7 +121,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -175,6 +175,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -301,7 +308,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -335,9 +342,6 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -347,10 +351,22 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -376,9 +392,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -416,7 +432,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -522,7 +538,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -664,7 +680,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -723,16 +739,16 @@
       <c r="B3" s="10">
         <v>90</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="15">
         <v>80</v>
       </c>
       <c r="D3" s="10">
         <v>80</v>
       </c>
-      <c r="E3" s="10">
+      <c r="E3" s="15">
         <v>70</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="16" t="s">
         <v>10</v>
       </c>
     </row>
@@ -740,19 +756,19 @@
       <c r="A4" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="11">
         <v>0</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="17">
         <v>60</v>
       </c>
-      <c r="D4" s="12">
+      <c r="D4" s="17">
         <v>120</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="17">
         <v>160</v>
       </c>
-      <c r="F4" s="13">
+      <c r="F4" s="12">
         <v>160</v>
       </c>
     </row>
@@ -763,16 +779,16 @@
       <c r="B5" s="10">
         <v>0</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="15">
         <v>-130</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="15">
         <v>-170</v>
       </c>
       <c r="E5" s="10">
         <v>-170</v>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="16">
         <v>-160</v>
       </c>
     </row>
@@ -780,30 +796,30 @@
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="14">
+      <c r="B6" s="13">
         <v>-150</v>
       </c>
-      <c r="C6" s="14">
+      <c r="C6" s="18">
         <v>-90</v>
       </c>
-      <c r="D6" s="14">
+      <c r="D6" s="18">
         <v>-45</v>
       </c>
-      <c r="E6" s="14">
+      <c r="E6" s="13">
         <v>-45</v>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="19">
         <v>-170</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="18.75" customHeight="1">
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>